<commit_message>
feat: pilot extraction of five papers into the template
Adds range fields to the cost table (value_min, value_max,
labour_days_min, labour_days_max) and an extractions/ folder with one CSV
per template sheet. Five African papers from the 2022 World Bank NbS
extraction are re-extracted: 118 effects, 118 cost rows, 161 quotes, all
found on their cited page (check A); 19 quotes checked for support (check
B). The comparison with the 2022 rows and the lessons for the template are
in extractions/README.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/synthesis/extraction_template.xlsx
+++ b/docs/synthesis/extraction_template.xlsx
@@ -3207,14 +3207,44 @@
             <color rgb="FF000000"/>
             <rFont val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">[CORE for pilots] [required] number
-As reported
+          <t xml:space="preserve">[CORE for pilots] [conditional] number
+As reported. Required unless the source gives a range, then value_min and value_max instead
 Allowed/unit: 
 Lands in: cost table</t>
         </r>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">[conditional] number
+Lower end, when the source gives a range (for example 1 in '1-26 person-days'). Leave value empty
+Allowed/unit: 
+Lands in: cost table</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">[conditional] number
+Upper end of a range. Filled with value_min
+Allowed/unit: 
+Lands in: cost table</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3229,7 +3259,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
+    <comment ref="M1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3244,7 +3274,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
+    <comment ref="N1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3259,7 +3289,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
+    <comment ref="O1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3273,7 +3303,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
+    <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3288,7 +3318,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
+    <comment ref="Q1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3297,13 +3327,43 @@
             <rFont val="Tahoma"/>
           </rPr>
           <t xml:space="preserve">[conditional] number
-Required if reported
+Required if reported, unless the source gives a range
 Allowed/unit: person-days per unit_basis
 Lands in: cost table</t>
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
+    <comment ref="R1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">[conditional] number
+Lower end when labour is reported as a range. Leave labour_days empty
+Allowed/unit: person-days per unit_basis
+Lands in: cost table</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">[conditional] number
+Upper end of a labour range
+Allowed/unit: person-days per unit_basis
+Lands in: cost table</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="T1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3318,7 +3378,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0" shapeId="0">
+    <comment ref="U1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3333,7 +3393,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R1" authorId="0" shapeId="0">
+    <comment ref="V1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3348,7 +3408,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S1" authorId="0" shapeId="0">
+    <comment ref="W1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3362,7 +3422,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T1" authorId="0" shapeId="0">
+    <comment ref="X1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3377,7 +3437,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
+    <comment ref="Y1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3392,7 +3452,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="V1" authorId="0" shapeId="0">
+    <comment ref="Z1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3407,7 +3467,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="W1" authorId="0" shapeId="0">
+    <comment ref="AA1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3422,7 +3482,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X1" authorId="0" shapeId="0">
+    <comment ref="AB1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3437,7 +3497,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Y1" authorId="0" shapeId="0">
+    <comment ref="AC1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3452,7 +3512,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z1" authorId="0" shapeId="0">
+    <comment ref="AD1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3467,7 +3527,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AA1" authorId="0" shapeId="0">
+    <comment ref="AE1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3482,7 +3542,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB1" authorId="0" shapeId="0">
+    <comment ref="AF1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3497,7 +3557,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AC1" authorId="0" shapeId="0">
+    <comment ref="AG1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3512,7 +3572,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AD1" authorId="0" shapeId="0">
+    <comment ref="AH1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3527,7 +3587,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AE1" authorId="0" shapeId="0">
+    <comment ref="AI1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3542,7 +3602,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AF1" authorId="0" shapeId="0">
+    <comment ref="AJ1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3557,7 +3617,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AG1" authorId="0" shapeId="0">
+    <comment ref="AK1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3572,7 +3632,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AH1" authorId="0" shapeId="0">
+    <comment ref="AL1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3587,7 +3647,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AI1" authorId="0" shapeId="0">
+    <comment ref="AM1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3602,7 +3662,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AJ1" authorId="0" shapeId="0">
+    <comment ref="AN1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3617,7 +3677,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AK1" authorId="0" shapeId="0">
+    <comment ref="AO1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -3632,7 +3692,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AL1" authorId="0" shapeId="0">
+    <comment ref="AP1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -4028,7 +4088,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="489">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="493">
   <si>
     <t xml:space="preserve">Extraction template, Activity 2 evidence synthesis (INV-089367)</t>
   </si>
@@ -4336,6 +4396,12 @@
     <t xml:space="preserve">value</t>
   </si>
   <si>
+    <t xml:space="preserve">value_min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value_max</t>
+  </si>
+  <si>
     <t xml:space="preserve">unit_basis</t>
   </si>
   <si>
@@ -4352,6 +4418,12 @@
   </si>
   <si>
     <t xml:space="preserve">labour_days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">labour_days_min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">labour_days_max</t>
   </si>
   <si>
     <t xml:space="preserve">labour_rate</t>
@@ -5931,7 +6003,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>6</v>
@@ -5940,67 +6012,67 @@
         <v>17</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>57</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="O1" s="2" t="s">
         <v>101</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="W1" s="3" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="X1" s="4" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -6098,7 +6170,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>6</v>
@@ -6110,31 +6182,31 @@
         <v>22</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -6200,7 +6272,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>6</v>
@@ -6209,28 +6281,28 @@
         <v>17</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>22</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>57</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -6299,64 +6371,64 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>23</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -6428,37 +6500,37 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>6</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
     </row>
   </sheetData>
@@ -6509,43 +6581,43 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="N1" s="4" t="s">
         <v>14</v>
@@ -6610,25 +6682,25 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>91</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -6669,1345 +6741,1345 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="B1" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C1" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="D1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E1" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="F1" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="G1" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="H1" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="I1" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="J1" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="K1" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="L1" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="M1" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="N1" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="O1" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="P1" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="Q1" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="R1" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="S1" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="T1" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="U1" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="V1" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="W1" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="X1" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="Y1" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="Z1" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="AA1" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="AB1" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="AC1" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="AD1" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AE1" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="AF1" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="AG1" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="AH1" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="AI1" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="AJ1" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AK1" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AL1" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AM1" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AN1" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="AO1" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AP1" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AQ1" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AR1" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="AS1" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="AT1" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="AU1" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="AV1" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="AW1" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="AX1" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="AY1" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="AZ1" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="BA1" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="BB1" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="BC1" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="BD1" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="BE1" t="s">
+        <v>404</v>
+      </c>
+      <c r="BF1" t="s">
+        <v>408</v>
+      </c>
+      <c r="BG1" t="s">
+        <v>412</v>
+      </c>
+      <c r="BH1" t="s">
+        <v>414</v>
+      </c>
+      <c r="BI1" t="s">
+        <v>418</v>
+      </c>
+      <c r="BJ1" t="s">
+        <v>423</v>
+      </c>
+      <c r="BK1" t="s">
+        <v>414</v>
+      </c>
+      <c r="BL1" t="s">
+        <v>237</v>
+      </c>
+      <c r="BM1" t="s">
+        <v>430</v>
+      </c>
+      <c r="BN1" t="s">
+        <v>267</v>
+      </c>
+      <c r="BO1" t="s">
+        <v>437</v>
+      </c>
+      <c r="BP1" t="s">
+        <v>267</v>
+      </c>
+      <c r="BQ1" t="s">
+        <v>237</v>
+      </c>
+      <c r="BR1" t="s">
+        <v>442</v>
+      </c>
+      <c r="BS1" t="s">
+        <v>445</v>
+      </c>
+      <c r="BT1" t="s">
+        <v>372</v>
+      </c>
+      <c r="BU1" t="s">
+        <v>267</v>
+      </c>
+      <c r="BV1" t="s">
+        <v>267</v>
+      </c>
+      <c r="BW1" t="s">
+        <v>267</v>
+      </c>
+      <c r="BX1" t="s">
+        <v>267</v>
+      </c>
+      <c r="BY1" t="s">
+        <v>449</v>
+      </c>
+      <c r="BZ1" t="s">
+        <v>272</v>
+      </c>
+      <c r="CA1" t="s">
+        <v>205</v>
+      </c>
+      <c r="CB1" t="s">
+        <v>455</v>
+      </c>
+      <c r="CC1" t="s">
         <v>400</v>
       </c>
-      <c r="BF1" t="s">
-        <v>404</v>
-      </c>
-      <c r="BG1" t="s">
-        <v>408</v>
-      </c>
-      <c r="BH1" t="s">
-        <v>410</v>
-      </c>
-      <c r="BI1" t="s">
-        <v>414</v>
-      </c>
-      <c r="BJ1" t="s">
-        <v>419</v>
-      </c>
-      <c r="BK1" t="s">
-        <v>410</v>
-      </c>
-      <c r="BL1" t="s">
-        <v>233</v>
-      </c>
-      <c r="BM1" t="s">
-        <v>426</v>
-      </c>
-      <c r="BN1" t="s">
-        <v>263</v>
-      </c>
-      <c r="BO1" t="s">
-        <v>433</v>
-      </c>
-      <c r="BP1" t="s">
-        <v>263</v>
-      </c>
-      <c r="BQ1" t="s">
-        <v>233</v>
-      </c>
-      <c r="BR1" t="s">
-        <v>438</v>
-      </c>
-      <c r="BS1" t="s">
-        <v>441</v>
-      </c>
-      <c r="BT1" t="s">
-        <v>368</v>
-      </c>
-      <c r="BU1" t="s">
-        <v>263</v>
-      </c>
-      <c r="BV1" t="s">
-        <v>263</v>
-      </c>
-      <c r="BW1" t="s">
-        <v>263</v>
-      </c>
-      <c r="BX1" t="s">
-        <v>263</v>
-      </c>
-      <c r="BY1" t="s">
-        <v>445</v>
-      </c>
-      <c r="BZ1" t="s">
-        <v>268</v>
-      </c>
-      <c r="CA1" t="s">
-        <v>201</v>
-      </c>
-      <c r="CB1" t="s">
-        <v>451</v>
-      </c>
-      <c r="CC1" t="s">
-        <v>396</v>
-      </c>
       <c r="CD1" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="CE1" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="CF1" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="CG1" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="CH1" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="CI1" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="CJ1" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="B2" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="C2" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="D2" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="E2" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="F2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="G2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="H2" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="I2" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="J2" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="K2" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="L2" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="M2" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="N2" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="O2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="P2" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="Q2" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="R2" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="S2" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="T2" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="U2" t="s">
+        <v>299</v>
+      </c>
+      <c r="V2" t="s">
+        <v>303</v>
+      </c>
+      <c r="W2" t="s">
+        <v>292</v>
+      </c>
+      <c r="X2" t="s">
+        <v>309</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>322</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>327</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>331</v>
+      </c>
+      <c r="AB2" t="s">
         <v>295</v>
       </c>
-      <c r="V2" t="s">
-        <v>299</v>
-      </c>
-      <c r="W2" t="s">
-        <v>288</v>
-      </c>
-      <c r="X2" t="s">
-        <v>305</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>318</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>323</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>327</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>291</v>
-      </c>
       <c r="AC2" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="AD2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AE2" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="AF2" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="AG2" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="AH2" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="AI2" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="AJ2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AK2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AL2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AM2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AN2" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="AO2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AP2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AQ2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AR2" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="AS2" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="AT2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="AU2" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="AV2" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="AW2" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="AX2" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="AY2" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="AZ2" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="BA2" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="BB2" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="BC2" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="BD2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="BE2" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="BF2" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="BG2" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="BH2" t="s">
         <v>98</v>
       </c>
       <c r="BI2" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="BJ2" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="BK2" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="BL2" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="BM2" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="BN2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="BO2" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
       <c r="BP2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="BQ2" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="BR2" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="BS2" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="BT2" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="BU2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="BV2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="BW2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="BX2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="BY2" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="BZ2" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="CA2" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="CB2" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="CC2" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="CD2" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="CE2" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="CF2" t="s">
-        <v>464</v>
+        <v>468</v>
       </c>
       <c r="CG2" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="CH2" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="CI2" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="CJ2" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="B3" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="C3" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="D3" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="E3" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="F3" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="G3" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="H3" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="I3" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="J3" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="K3" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="L3" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="M3" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="N3" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="O3" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="P3" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="Q3" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="R3" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="S3" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="T3" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="U3" t="s">
+        <v>300</v>
+      </c>
+      <c r="V3" t="s">
+        <v>304</v>
+      </c>
+      <c r="W3" t="s">
+        <v>307</v>
+      </c>
+      <c r="X3" t="s">
+        <v>310</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>323</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>328</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>332</v>
+      </c>
+      <c r="AB3" t="s">
         <v>296</v>
       </c>
-      <c r="V3" t="s">
-        <v>300</v>
-      </c>
-      <c r="W3" t="s">
-        <v>303</v>
-      </c>
-      <c r="X3" t="s">
-        <v>306</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>319</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>324</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>328</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>292</v>
-      </c>
       <c r="AC3" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="AD3" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="AE3" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="AF3" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="AG3" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="AH3" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="AI3" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="AJ3" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="AK3" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="AL3" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="AM3" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="AN3" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="AO3" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="AP3" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="AQ3" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="AR3" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="AS3" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="AU3" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="AW3" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="AX3" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="AY3" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="AZ3" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="BA3" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="BB3" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="BC3" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="BD3" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="BE3" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="BF3" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="BG3" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="BH3" t="s">
+        <v>415</v>
+      </c>
+      <c r="BI3" t="s">
+        <v>420</v>
+      </c>
+      <c r="BJ3" t="s">
+        <v>425</v>
+      </c>
+      <c r="BK3" t="s">
+        <v>429</v>
+      </c>
+      <c r="BL3" t="s">
+        <v>239</v>
+      </c>
+      <c r="BM3" t="s">
+        <v>432</v>
+      </c>
+      <c r="BO3" t="s">
+        <v>439</v>
+      </c>
+      <c r="BP3" t="s">
+        <v>281</v>
+      </c>
+      <c r="BQ3" t="s">
+        <v>239</v>
+      </c>
+      <c r="BR3" t="s">
+        <v>444</v>
+      </c>
+      <c r="BS3" t="s">
+        <v>276</v>
+      </c>
+      <c r="BT3" t="s">
         <v>411</v>
       </c>
-      <c r="BI3" t="s">
-        <v>416</v>
-      </c>
-      <c r="BJ3" t="s">
-        <v>421</v>
-      </c>
-      <c r="BK3" t="s">
-        <v>425</v>
-      </c>
-      <c r="BL3" t="s">
-        <v>235</v>
-      </c>
-      <c r="BM3" t="s">
-        <v>428</v>
-      </c>
-      <c r="BO3" t="s">
-        <v>435</v>
-      </c>
-      <c r="BP3" t="s">
-        <v>277</v>
-      </c>
-      <c r="BQ3" t="s">
-        <v>235</v>
-      </c>
-      <c r="BR3" t="s">
-        <v>440</v>
-      </c>
-      <c r="BS3" t="s">
-        <v>272</v>
-      </c>
-      <c r="BT3" t="s">
-        <v>407</v>
-      </c>
       <c r="BU3" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="BV3" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="BW3" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="BX3" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="BY3" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="BZ3" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="CA3" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="CB3" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="CC3" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="CD3" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="CE3" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="CF3" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="CG3" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="CH3" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="CI3" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="CJ3" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="B4" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="C4" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="D4" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="E4" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="H4" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="I4" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="J4" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="K4" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="L4" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="M4" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="N4" t="s">
+        <v>280</v>
+      </c>
+      <c r="P4" t="s">
+        <v>281</v>
+      </c>
+      <c r="Q4" t="s">
         <v>276</v>
       </c>
-      <c r="P4" t="s">
-        <v>277</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>272</v>
-      </c>
       <c r="T4" t="s">
+        <v>297</v>
+      </c>
+      <c r="U4" t="s">
+        <v>301</v>
+      </c>
+      <c r="V4" t="s">
+        <v>305</v>
+      </c>
+      <c r="W4" t="s">
         <v>293</v>
       </c>
-      <c r="U4" t="s">
+      <c r="X4" t="s">
+        <v>311</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>324</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>329</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>333</v>
+      </c>
+      <c r="AB4" t="s">
         <v>297</v>
       </c>
-      <c r="V4" t="s">
-        <v>301</v>
-      </c>
-      <c r="W4" t="s">
-        <v>289</v>
-      </c>
-      <c r="X4" t="s">
-        <v>307</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>320</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>325</v>
-      </c>
-      <c r="AA4" t="s">
-        <v>329</v>
-      </c>
-      <c r="AB4" t="s">
+      <c r="AF4" t="s">
+        <v>240</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>343</v>
+      </c>
+      <c r="AH4" t="s">
+        <v>354</v>
+      </c>
+      <c r="AN4" t="s">
+        <v>268</v>
+      </c>
+      <c r="AR4" t="s">
+        <v>367</v>
+      </c>
+      <c r="AS4" t="s">
+        <v>276</v>
+      </c>
+      <c r="AU4" t="s">
+        <v>376</v>
+      </c>
+      <c r="AW4" t="s">
+        <v>387</v>
+      </c>
+      <c r="AX4" t="s">
+        <v>297</v>
+      </c>
+      <c r="AZ4" t="s">
+        <v>391</v>
+      </c>
+      <c r="BA4" t="s">
+        <v>396</v>
+      </c>
+      <c r="BB4" t="s">
+        <v>240</v>
+      </c>
+      <c r="BC4" t="s">
+        <v>403</v>
+      </c>
+      <c r="BE4" t="s">
+        <v>407</v>
+      </c>
+      <c r="BF4" t="s">
+        <v>411</v>
+      </c>
+      <c r="BH4" t="s">
+        <v>416</v>
+      </c>
+      <c r="BI4" t="s">
+        <v>421</v>
+      </c>
+      <c r="BJ4" t="s">
+        <v>426</v>
+      </c>
+      <c r="BK4" t="s">
         <v>293</v>
       </c>
-      <c r="AF4" t="s">
-        <v>236</v>
-      </c>
-      <c r="AG4" t="s">
+      <c r="BL4" t="s">
+        <v>240</v>
+      </c>
+      <c r="BM4" t="s">
+        <v>433</v>
+      </c>
+      <c r="BO4" t="s">
+        <v>440</v>
+      </c>
+      <c r="BQ4" t="s">
+        <v>240</v>
+      </c>
+      <c r="BR4" t="s">
+        <v>281</v>
+      </c>
+      <c r="BS4" t="s">
+        <v>281</v>
+      </c>
+      <c r="BT4" t="s">
+        <v>448</v>
+      </c>
+      <c r="BY4" t="s">
+        <v>293</v>
+      </c>
+      <c r="CB4" t="s">
+        <v>457</v>
+      </c>
+      <c r="CC4" t="s">
+        <v>461</v>
+      </c>
+      <c r="CD4" t="s">
         <v>339</v>
       </c>
-      <c r="AH4" t="s">
-        <v>350</v>
-      </c>
-      <c r="AN4" t="s">
-        <v>264</v>
-      </c>
-      <c r="AR4" t="s">
-        <v>363</v>
-      </c>
-      <c r="AS4" t="s">
-        <v>272</v>
-      </c>
-      <c r="AU4" t="s">
-        <v>372</v>
-      </c>
-      <c r="AW4" t="s">
-        <v>383</v>
-      </c>
-      <c r="AX4" t="s">
-        <v>293</v>
-      </c>
-      <c r="AZ4" t="s">
-        <v>387</v>
-      </c>
-      <c r="BA4" t="s">
-        <v>392</v>
-      </c>
-      <c r="BB4" t="s">
-        <v>236</v>
-      </c>
-      <c r="BC4" t="s">
-        <v>399</v>
-      </c>
-      <c r="BE4" t="s">
-        <v>403</v>
-      </c>
-      <c r="BF4" t="s">
-        <v>407</v>
-      </c>
-      <c r="BH4" t="s">
-        <v>412</v>
-      </c>
-      <c r="BI4" t="s">
-        <v>417</v>
-      </c>
-      <c r="BJ4" t="s">
-        <v>422</v>
-      </c>
-      <c r="BK4" t="s">
-        <v>289</v>
-      </c>
-      <c r="BL4" t="s">
-        <v>236</v>
-      </c>
-      <c r="BM4" t="s">
-        <v>429</v>
-      </c>
-      <c r="BO4" t="s">
-        <v>436</v>
-      </c>
-      <c r="BQ4" t="s">
-        <v>236</v>
-      </c>
-      <c r="BR4" t="s">
-        <v>277</v>
-      </c>
-      <c r="BS4" t="s">
-        <v>277</v>
-      </c>
-      <c r="BT4" t="s">
-        <v>444</v>
-      </c>
-      <c r="BY4" t="s">
-        <v>289</v>
-      </c>
-      <c r="CB4" t="s">
-        <v>453</v>
-      </c>
-      <c r="CC4" t="s">
-        <v>457</v>
-      </c>
-      <c r="CD4" t="s">
-        <v>335</v>
-      </c>
       <c r="CF4" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="CG4" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="CH4" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="CI4" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="CJ4" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="B5" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="C5" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="D5" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="T5" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="V5" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="X5" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="Y5" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="AB5" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="AF5" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="AG5" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="AH5" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="AN5" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="AR5" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="AS5" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="AU5" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="AX5" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="AZ5" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="BA5" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="BB5" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="BH5" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
       <c r="BI5" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="BJ5" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="BL5" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="BM5" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="BO5" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="BQ5" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="CB5" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="CF5" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="CH5" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="CI5" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="B6" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="D6" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="X6" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="Y6" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="AF6" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="AG6" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="AH6" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="AR6" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="AU6" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="BA6" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="BB6" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="BJ6" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="BL6" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="BM6" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="BO6" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="BQ6" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="CB6" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="CF6" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="CH6" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="CI6" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B7" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="D7" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="X7" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="AF7" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="AG7" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AH7" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="AU7" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="BA7" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
       <c r="BB7" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="BJ7" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="BL7" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="BM7" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="BQ7" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="CF7" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="CI7" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="B8" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="D8" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="X8" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="AF8" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="AG8" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="AU8" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="BB8" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="BL8" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="BM8" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="BQ8" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="CF8" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="CI8" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="D9" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="X9" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="AF9" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="AG9" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="AU9" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="BB9" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="BL9" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="BQ9" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="CF9" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="CI9" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="D10" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="X10" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="AF10" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="AG10" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="BB10" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="BL10" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="BQ10" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="CF10" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="X11" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="AF11" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="AG11" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="BB11" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="BL11" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="BQ11" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="X12" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="AF12" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="BB12" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="BL12" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="BQ12" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="X13" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="AF13" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="BB13" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="BL13" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="BQ13" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
   </sheetData>
@@ -8714,35 +8786,39 @@
     <col min="7" max="7" width="14.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="13.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="13.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="14.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="13.71" hidden="0" customWidth="1"/>
     <col min="11" max="11" width="13.71" hidden="0" customWidth="1"/>
     <col min="12" max="12" width="14.71" hidden="0" customWidth="1"/>
-    <col min="13" max="13" width="20.71" hidden="0" customWidth="1"/>
-    <col min="14" max="14" width="19.71" hidden="0" customWidth="1"/>
-    <col min="15" max="15" width="15.71" hidden="0" customWidth="1"/>
-    <col min="16" max="16" width="15.71" hidden="0" customWidth="1"/>
-    <col min="17" max="17" width="24.71" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="13.71" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="14.71" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="20.71" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="19.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="15.71" hidden="0" customWidth="1"/>
     <col min="18" max="18" width="19.71" hidden="0" customWidth="1"/>
-    <col min="19" max="19" width="22.71" hidden="0" customWidth="1"/>
-    <col min="20" max="20" width="22.71" hidden="0" customWidth="1"/>
-    <col min="21" max="21" width="21.71" hidden="0" customWidth="1"/>
-    <col min="22" max="22" width="30.71" hidden="0" customWidth="1"/>
-    <col min="23" max="23" width="29.71" hidden="0" customWidth="1"/>
-    <col min="24" max="24" width="17.71" hidden="0" customWidth="1"/>
-    <col min="25" max="25" width="17.71" hidden="0" customWidth="1"/>
-    <col min="26" max="26" width="21.71" hidden="0" customWidth="1"/>
-    <col min="27" max="27" width="17.71" hidden="0" customWidth="1"/>
+    <col min="19" max="19" width="19.71" hidden="0" customWidth="1"/>
+    <col min="20" max="20" width="15.71" hidden="0" customWidth="1"/>
+    <col min="21" max="21" width="24.71" hidden="0" customWidth="1"/>
+    <col min="22" max="22" width="19.71" hidden="0" customWidth="1"/>
+    <col min="23" max="23" width="22.71" hidden="0" customWidth="1"/>
+    <col min="24" max="24" width="22.71" hidden="0" customWidth="1"/>
+    <col min="25" max="25" width="21.71" hidden="0" customWidth="1"/>
+    <col min="26" max="26" width="30.71" hidden="0" customWidth="1"/>
+    <col min="27" max="27" width="29.71" hidden="0" customWidth="1"/>
     <col min="28" max="28" width="17.71" hidden="0" customWidth="1"/>
-    <col min="29" max="29" width="21.71" hidden="0" customWidth="1"/>
-    <col min="30" max="30" width="19.71" hidden="0" customWidth="1"/>
-    <col min="31" max="31" width="16.71" hidden="0" customWidth="1"/>
-    <col min="32" max="32" width="26.71" hidden="0" customWidth="1"/>
-    <col min="33" max="33" width="24.71" hidden="0" customWidth="1"/>
-    <col min="34" max="34" width="15.71" hidden="0" customWidth="1"/>
-    <col min="35" max="35" width="19.71" hidden="0" customWidth="1"/>
-    <col min="36" max="36" width="17.71" hidden="0" customWidth="1"/>
-    <col min="37" max="37" width="17.71" hidden="0" customWidth="1"/>
-    <col min="38" max="38" width="21.71" hidden="0" customWidth="1"/>
+    <col min="29" max="29" width="17.71" hidden="0" customWidth="1"/>
+    <col min="30" max="30" width="21.71" hidden="0" customWidth="1"/>
+    <col min="31" max="31" width="17.71" hidden="0" customWidth="1"/>
+    <col min="32" max="32" width="17.71" hidden="0" customWidth="1"/>
+    <col min="33" max="33" width="21.71" hidden="0" customWidth="1"/>
+    <col min="34" max="34" width="19.71" hidden="0" customWidth="1"/>
+    <col min="35" max="35" width="16.71" hidden="0" customWidth="1"/>
+    <col min="36" max="36" width="26.71" hidden="0" customWidth="1"/>
+    <col min="37" max="37" width="24.71" hidden="0" customWidth="1"/>
+    <col min="38" max="38" width="15.71" hidden="0" customWidth="1"/>
+    <col min="39" max="39" width="19.71" hidden="0" customWidth="1"/>
+    <col min="40" max="40" width="17.71" hidden="0" customWidth="1"/>
+    <col min="41" max="41" width="17.71" hidden="0" customWidth="1"/>
+    <col min="42" max="42" width="21.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8770,13 +8846,13 @@
       <c r="H1" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="3" t="s">
         <v>103</v>
       </c>
       <c r="L1" s="2" t="s">
@@ -8788,22 +8864,22 @@
       <c r="N1" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="P1" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="3" t="s">
         <v>112</v>
       </c>
       <c r="U1" s="2" t="s">
@@ -8815,28 +8891,28 @@
       <c r="W1" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="X1" s="4" t="s">
+      <c r="X1" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="Y1" s="4" t="s">
+      <c r="Y1" s="2" t="s">
         <v>117</v>
       </c>
       <c r="Z1" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="AA1" s="4" t="s">
+      <c r="AA1" s="2" t="s">
         <v>119</v>
       </c>
       <c r="AB1" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AC1" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="AD1" s="3" t="s">
+      <c r="AD1" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="AE1" s="3" t="s">
+      <c r="AE1" s="4" t="s">
         <v>123</v>
       </c>
       <c r="AF1" s="4" t="s">
@@ -8845,13 +8921,13 @@
       <c r="AG1" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AH1" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="AI1" s="2" t="s">
+      <c r="AI1" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="AJ1" s="3" t="s">
+      <c r="AJ1" s="4" t="s">
         <v>128</v>
       </c>
       <c r="AK1" s="3" t="s">
@@ -8859,6 +8935,18 @@
       </c>
       <c r="AL1" s="2" t="s">
         <v>130</v>
+      </c>
+      <c r="AM1" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="AN1" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="AO1" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="AP1" s="2" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -8884,79 +8972,79 @@
           <x14:formula1>
             <xm:f>'_lists'!$AH$1:$AH$7</xm:f>
           </x14:formula1>
-          <xm:sqref>J2:J2001</xm:sqref>
+          <xm:sqref>L2:L2001</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0">
           <x14:formula1>
             <xm:f>'_lists'!$AI$1:$AI$3</xm:f>
           </x14:formula1>
-          <xm:sqref>M2:M2001</xm:sqref>
+          <xm:sqref>O2:O2001</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0">
           <x14:formula1>
             <xm:f>'_lists'!$AJ$1:$AJ$3</xm:f>
           </x14:formula1>
-          <xm:sqref>N2:N2001</xm:sqref>
+          <xm:sqref>P2:P2001</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0">
           <x14:formula1>
             <xm:f>'_lists'!$AK$1:$AK$3</xm:f>
           </x14:formula1>
-          <xm:sqref>Q2:Q2001</xm:sqref>
+          <xm:sqref>U2:U2001</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0">
           <x14:formula1>
             <xm:f>'_lists'!$AL$1:$AL$3</xm:f>
           </x14:formula1>
-          <xm:sqref>R2:R2001</xm:sqref>
+          <xm:sqref>V2:V2001</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0">
           <x14:formula1>
             <xm:f>'_lists'!$AM$1:$AM$3</xm:f>
           </x14:formula1>
-          <xm:sqref>S2:S2001</xm:sqref>
+          <xm:sqref>W2:W2001</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0">
           <x14:formula1>
             <xm:f>'_lists'!$AN$1:$AN$5</xm:f>
           </x14:formula1>
-          <xm:sqref>T2:T2001</xm:sqref>
+          <xm:sqref>X2:X2001</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0">
           <x14:formula1>
             <xm:f>'_lists'!$AO$1:$AO$3</xm:f>
           </x14:formula1>
-          <xm:sqref>U2:U2001</xm:sqref>
+          <xm:sqref>Y2:Y2001</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0">
           <x14:formula1>
             <xm:f>'_lists'!$AP$1:$AP$3</xm:f>
           </x14:formula1>
-          <xm:sqref>V2:V2001</xm:sqref>
+          <xm:sqref>Z2:Z2001</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0">
           <x14:formula1>
             <xm:f>'_lists'!$AQ$1:$AQ$3</xm:f>
           </x14:formula1>
-          <xm:sqref>W2:W2001</xm:sqref>
+          <xm:sqref>AA2:AA2001</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0">
           <x14:formula1>
             <xm:f>'_lists'!$AR$1:$AR$6</xm:f>
           </x14:formula1>
-          <xm:sqref>Z2:Z2001</xm:sqref>
+          <xm:sqref>AD2:AD2001</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0">
           <x14:formula1>
             <xm:f>'_lists'!$AS$1:$AS$5</xm:f>
           </x14:formula1>
-          <xm:sqref>AH2:AH2001</xm:sqref>
+          <xm:sqref>AL2:AL2001</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0">
           <x14:formula1>
             <xm:f>'_lists'!$AT$1:$AT$2</xm:f>
           </x14:formula1>
-          <xm:sqref>AI2:AI2001</xm:sqref>
+          <xm:sqref>AM2:AM2001</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -8980,7 +9068,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>6</v>
@@ -8989,7 +9077,7 @@
         <v>15</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>101</v>
@@ -8998,7 +9086,7 @@
         <v>79</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -9046,55 +9134,55 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>6</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>78</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>91</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>71</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="L1" s="2" t="s">
         <v>57</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>